<commit_message>
Feat: Audiotria general y pdf
</commit_message>
<xml_diff>
--- a/outputs/grupo3_entrega_grupo7.xlsx
+++ b/outputs/grupo3_entrega_grupo7.xlsx
@@ -2680,10 +2680,10 @@
         <v>1643.180665894866</v>
       </c>
       <c r="H5" t="n">
-        <v>1594.583641586144</v>
+        <v>1594.583641586143</v>
       </c>
       <c r="I5" t="n">
-        <v>1691.777690203588</v>
+        <v>1691.777690203589</v>
       </c>
       <c r="J5" t="n">
         <v>1643.180665894866</v>
@@ -6397,10 +6397,10 @@
         <v>59.61669133026552</v>
       </c>
       <c r="L70" t="n">
-        <v>57.63409903622372</v>
+        <v>57.63409903622371</v>
       </c>
       <c r="M70" t="n">
-        <v>61.59928362430733</v>
+        <v>61.59928362430734</v>
       </c>
       <c r="N70" t="n">
         <v>0</v>
@@ -7981,7 +7981,7 @@
         <v>1835.942429054067</v>
       </c>
       <c r="H98" t="n">
-        <v>1786.323334478552</v>
+        <v>1786.323334478551</v>
       </c>
       <c r="I98" t="n">
         <v>1885.561523629583</v>
@@ -8107,19 +8107,19 @@
         <v>4.842336225953686</v>
       </c>
       <c r="L100" t="n">
-        <v>3.509185671110904</v>
+        <v>3.509185671110903</v>
       </c>
       <c r="M100" t="n">
-        <v>6.175486780796469</v>
+        <v>6.17548678079647</v>
       </c>
       <c r="N100" t="n">
         <v>5.562649214081772</v>
       </c>
       <c r="O100" t="n">
-        <v>4.123540686377363</v>
+        <v>4.123540686377362</v>
       </c>
       <c r="P100" t="n">
-        <v>7.001757741786181</v>
+        <v>7.001757741786182</v>
       </c>
       <c r="Q100" t="n">
         <v>4.842336225953686</v>
@@ -8458,7 +8458,7 @@
         <v>0.07094680891075138</v>
       </c>
       <c r="O106" t="n">
-        <v>-0.02412281042554712</v>
+        <v>-0.02412281042554713</v>
       </c>
       <c r="P106" t="n">
         <v>0.1660164282470499</v>
@@ -9301,10 +9301,10 @@
         <v>12.72870780911049</v>
       </c>
       <c r="K121" t="n">
-        <v>1.275922973172919</v>
+        <v>1.275922973172918</v>
       </c>
       <c r="L121" t="n">
-        <v>0.7419283191298101</v>
+        <v>0.7419283191298097</v>
       </c>
       <c r="M121" t="n">
         <v>1.809917627216027</v>
@@ -9319,7 +9319,7 @@
         <v>7.345679093561179</v>
       </c>
       <c r="Q121" t="n">
-        <v>1.275922973172919</v>
+        <v>1.275922973172918</v>
       </c>
     </row>
     <row r="122">
@@ -9520,7 +9520,7 @@
         <v>1648.001820528082</v>
       </c>
       <c r="H125" t="n">
-        <v>1594.458905018865</v>
+        <v>1594.458905018864</v>
       </c>
       <c r="I125" t="n">
         <v>1701.5447360373</v>
@@ -10138,7 +10138,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>1.275922973172919</v>
+        <v>1.275922973172918</v>
       </c>
       <c r="F136" t="n">
         <v>0</v>
@@ -10159,7 +10159,7 @@
         <v>0.01040861832033949</v>
       </c>
       <c r="L136" t="n">
-        <v>-0.01024433859347106</v>
+        <v>-0.01024433859347107</v>
       </c>
       <c r="M136" t="n">
         <v>0.03106157523415004</v>
@@ -11116,10 +11116,10 @@
         <v>100.3791309146555</v>
       </c>
       <c r="H153" t="n">
-        <v>97.40116886244445</v>
+        <v>97.40116886244444</v>
       </c>
       <c r="I153" t="n">
-        <v>103.3570929668666</v>
+        <v>103.3570929668667</v>
       </c>
       <c r="J153" t="n">
         <v>0</v>
@@ -11137,10 +11137,10 @@
         <v>100.3791309146555</v>
       </c>
       <c r="O153" t="n">
-        <v>97.40116886244445</v>
+        <v>97.40116886244444</v>
       </c>
       <c r="P153" t="n">
-        <v>103.3570929668666</v>
+        <v>103.3570929668667</v>
       </c>
       <c r="Q153" t="n">
         <v>0</v>
@@ -11857,10 +11857,10 @@
         <v>18.28938190521779</v>
       </c>
       <c r="H166" t="n">
-        <v>17.80765114711978</v>
+        <v>17.80765114711977</v>
       </c>
       <c r="I166" t="n">
-        <v>18.7711126633158</v>
+        <v>18.77111266331581</v>
       </c>
       <c r="J166" t="n">
         <v>0</v>
@@ -11878,10 +11878,10 @@
         <v>18.28938190521779</v>
       </c>
       <c r="O166" t="n">
-        <v>17.80765114711978</v>
+        <v>17.80765114711977</v>
       </c>
       <c r="P166" t="n">
-        <v>18.7711126633158</v>
+        <v>18.77111266331581</v>
       </c>
       <c r="Q166" t="n">
         <v>0</v>
@@ -12487,7 +12487,7 @@
         <v>507.0139914217811</v>
       </c>
       <c r="I177" t="n">
-        <v>537.199613355376</v>
+        <v>537.1996133553761</v>
       </c>
       <c r="J177" t="n">
         <v>522.1068023885786</v>
@@ -12670,7 +12670,7 @@
         <v>2658.289150510537</v>
       </c>
       <c r="M180" t="n">
-        <v>2735.841449225554</v>
+        <v>2735.841449225555</v>
       </c>
       <c r="N180" t="n">
         <v>0</v>
@@ -17622,7 +17622,7 @@
         <v>0.05092418369978944</v>
       </c>
       <c r="O85" t="n">
-        <v>-0.02383065911625998</v>
+        <v>-0.02383065911626</v>
       </c>
       <c r="P85" t="n">
         <v>0.1256790265158389</v>
@@ -17967,7 +17967,7 @@
         <v>0.161121439258964</v>
       </c>
       <c r="P91" t="n">
-        <v>0.8834333982098467</v>
+        <v>0.8834333982098468</v>
       </c>
       <c r="Q91" t="n">
         <v>10.96925877899999</v>
@@ -18303,10 +18303,10 @@
         <v>34.37774883932048</v>
       </c>
       <c r="N97" t="n">
-        <v>0.7629531739555643</v>
+        <v>0.7629531739555639</v>
       </c>
       <c r="O97" t="n">
-        <v>0.1340334502599468</v>
+        <v>0.1340334502599463</v>
       </c>
       <c r="P97" t="n">
         <v>1.391872897651182</v>
@@ -18462,7 +18462,7 @@
         <v>31.13453762632048</v>
       </c>
       <c r="J100" t="n">
-        <v>20.54960803790788</v>
+        <v>20.54960803790787</v>
       </c>
       <c r="K100" t="n">
         <v>2.392624606826031</v>
@@ -18807,13 +18807,13 @@
         <v>10.76078471975531</v>
       </c>
       <c r="K106" t="n">
-        <v>0.2084740592446749</v>
+        <v>0.2084740592446748</v>
       </c>
       <c r="L106" t="n">
-        <v>0.000910888200489457</v>
+        <v>0.0009108882004894847</v>
       </c>
       <c r="M106" t="n">
-        <v>0.4160372302888604</v>
+        <v>0.4160372302888601</v>
       </c>
       <c r="N106" t="n">
         <v>11.96577587246307</v>
@@ -18825,7 +18825,7 @@
         <v>13.42802615117904</v>
       </c>
       <c r="Q106" t="n">
-        <v>0.2084740592446749</v>
+        <v>0.2084740592446748</v>
       </c>
     </row>
     <row r="107">
@@ -19152,7 +19152,7 @@
         <v>1.968433072645277</v>
       </c>
       <c r="L112" t="n">
-        <v>0.9104874156749463</v>
+        <v>0.9104874156749461</v>
       </c>
       <c r="M112" t="n">
         <v>3.026378729615607</v>
@@ -19164,7 +19164,7 @@
         <v>17.41697578895135</v>
       </c>
       <c r="P112" t="n">
-        <v>24.89469101954966</v>
+        <v>24.89469101954967</v>
       </c>
       <c r="Q112" t="n">
         <v>1.968433072645277</v>
@@ -19314,7 +19314,7 @@
         <v>30.16689069705543</v>
       </c>
       <c r="I115" t="n">
-        <v>32.13825321385627</v>
+        <v>32.13825321385628</v>
       </c>
       <c r="J115" t="n">
         <v>2.392624606826031</v>
@@ -19644,7 +19644,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>0.2084740592446749</v>
+        <v>0.2084740592446748</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -19659,7 +19659,7 @@
         <v>23.37434620327786</v>
       </c>
       <c r="J121" t="n">
-        <v>0.2084740592446749</v>
+        <v>0.2084740592446748</v>
       </c>
       <c r="K121" t="n">
         <v>0</v>
@@ -20736,10 +20736,10 @@
         <v>3028.870379716927</v>
       </c>
       <c r="H140" t="n">
-        <v>2937.637913993965</v>
+        <v>2937.637913993964</v>
       </c>
       <c r="I140" t="n">
-        <v>3120.10284543989</v>
+        <v>3120.102845439891</v>
       </c>
       <c r="J140" t="n">
         <v>3028.870379716927</v>
@@ -21081,7 +21081,7 @@
         <v>7802.722435067236</v>
       </c>
       <c r="I146" t="n">
-        <v>8268.249827464491</v>
+        <v>8268.249827464493</v>
       </c>
       <c r="J146" t="n">
         <v>8035.486131265864</v>
@@ -22674,10 +22674,10 @@
         <v>633.956430840872</v>
       </c>
       <c r="H174" t="n">
-        <v>614.6712296782447</v>
+        <v>614.6712296782446</v>
       </c>
       <c r="I174" t="n">
-        <v>653.2416320034994</v>
+        <v>653.2416320034995</v>
       </c>
       <c r="J174" t="n">
         <v>633.956430840872</v>

</xml_diff>